<commit_message>
gene14: validate morphseq sequencing identity map
</commit_message>
<xml_diff>
--- a/results/mcolon/20260607_sci_cilia_gene14_imaging_qc/source_plate_metadata_excels/20260319_cilia_crispant_24hpf_well_metadata.xlsx
+++ b/results/mcolon/20260607_sci_cilia_gene14_imaging_qc/source_plate_metadata_excels/20260319_cilia_crispant_24hpf_well_metadata.xlsx
@@ -518,7 +518,11 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
           <t>A02</t>
@@ -561,8 +565,16 @@
           <t>B12</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="n"/>
@@ -600,8 +612,16 @@
           <t>C12</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
@@ -639,8 +659,16 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
@@ -678,8 +706,16 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
@@ -717,8 +753,16 @@
           <t>F12</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
@@ -756,8 +800,16 @@
           <t>G12</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
@@ -795,8 +847,16 @@
           <t>H12</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>H01</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>H02</t>
+        </is>
+      </c>
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
@@ -1135,374 +1195,374 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" t="n">
+      <c r="B1" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E1" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F1" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G1" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H1" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I1" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="J1" t="n">
+      <c r="J1" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="K1" t="n">
+      <c r="K1" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="L1" t="n">
+      <c r="L1" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="M1" t="n">
+      <c r="M1" s="0" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Bl1</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Bl1</t>
+        </is>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
         <is>
           <t>Bl1</t>
         </is>

</xml_diff>